<commit_message>
vimal time sheet update
</commit_message>
<xml_diff>
--- a/timesheet/vimal_timesheet.xlsx
+++ b/timesheet/vimal_timesheet.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="10">
   <si>
     <t>Date</t>
   </si>
@@ -42,6 +42,15 @@
   </si>
   <si>
     <t>researched 2 good and bad charts and pushed in git hub and gave brief discription</t>
+  </si>
+  <si>
+    <t>researched three sample questions and gave answer to it</t>
+  </si>
+  <si>
+    <t>learned excel sheet and made bad chart make ovet</t>
+  </si>
+  <si>
+    <t>researched online for bangalore rain fall data and collected it</t>
   </si>
   <si>
     <t/>
@@ -1275,8 +1284,8 @@
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>5</v>
+      <c r="C4" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1284,10 +1293,10 @@
         <v>46315</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1295,10 +1304,10 @@
         <v>46316</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="C6" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1306,10 +1315,10 @@
         <v>46317</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1322,10 +1331,10 @@
         <v>46319</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1333,10 +1342,10 @@
         <v>46320</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1344,10 +1353,10 @@
         <v>46321</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1355,10 +1364,10 @@
         <v>46322</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1366,10 +1375,10 @@
         <v>46323</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1377,10 +1386,10 @@
         <v>46324</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1388,10 +1397,10 @@
         <v>46325</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1399,10 +1408,10 @@
         <v>46326</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1410,10 +1419,10 @@
         <v>46327</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1421,10 +1430,10 @@
         <v>46328</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1432,10 +1441,10 @@
         <v>46329</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1443,10 +1452,10 @@
         <v>46330</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1454,10 +1463,10 @@
         <v>46331</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1465,10 +1474,10 @@
         <v>46332</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1476,10 +1485,10 @@
         <v>46333</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1487,10 +1496,10 @@
         <v>46334</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1498,10 +1507,10 @@
         <v>46335</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1509,10 +1518,10 @@
         <v>46336</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1520,10 +1529,10 @@
         <v>46337</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1531,10 +1540,10 @@
         <v>46338</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1542,10 +1551,10 @@
         <v>46339</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1553,10 +1562,10 @@
         <v>46340</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1564,10 +1573,10 @@
         <v>46341</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1575,10 +1584,10 @@
         <v>46342</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1586,20 +1595,20 @@
         <v>46343</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="4"/>
       <c r="B34" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C34" s="4">
         <f>SUM(C2:C33)</f>
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>